<commit_message>
fix probleme liaison entre plusieurs années et promotions et etudiants
</commit_message>
<xml_diff>
--- a/fichiers_test/etudiants_FIE3_2025-26_S6.xlsx
+++ b/fichiers_test/etudiants_FIE3_2025-26_S6.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="137">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -38,6 +38,9 @@
   </si>
   <si>
     <t xml:space="preserve">lv2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">annee_debut</t>
   </si>
   <si>
     <t xml:space="preserve">eya.abid_ghozzi@etud.univ-jfc.fr</t>
@@ -782,7 +785,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
@@ -812,25 +815,31 @@
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="0" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G2" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -838,19 +847,22 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G3" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -858,19 +870,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G4" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -878,19 +893,22 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G5" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -898,19 +916,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G6" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -918,19 +939,22 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G7" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -938,19 +962,22 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G8" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -958,19 +985,22 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G9" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -978,19 +1008,22 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G10" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -998,19 +1031,22 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G11" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1018,19 +1054,22 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G12" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1038,19 +1077,22 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G13" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1058,19 +1100,22 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G14" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1078,19 +1123,22 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G15" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1098,19 +1146,22 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G16" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1118,19 +1169,22 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G17" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1138,19 +1192,22 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G18" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1158,19 +1215,22 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G19" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1178,19 +1238,22 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G20" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1198,19 +1261,22 @@
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G21" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1218,19 +1284,22 @@
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G22" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1238,19 +1307,22 @@
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G23" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1258,19 +1330,22 @@
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G24" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1278,19 +1353,22 @@
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G25" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1298,19 +1376,22 @@
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G26" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1318,19 +1399,22 @@
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G27" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1338,19 +1422,22 @@
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G28" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1358,19 +1445,22 @@
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G29" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1378,19 +1468,22 @@
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G30" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1398,19 +1491,22 @@
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G31" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1418,19 +1514,22 @@
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G32" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1438,19 +1537,22 @@
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G33" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1458,19 +1560,22 @@
         <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G34" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1478,19 +1583,22 @@
         <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G35" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1498,19 +1606,22 @@
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G36" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1518,19 +1629,22 @@
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G37" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1538,19 +1652,22 @@
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G38" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1558,19 +1675,22 @@
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G39" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1578,19 +1698,22 @@
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="G40" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1598,19 +1721,22 @@
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G41" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1618,19 +1744,22 @@
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G42" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1638,19 +1767,22 @@
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G43" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1658,19 +1790,22 @@
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="G44" s="0" t="n">
+        <v>2025</v>
       </c>
     </row>
   </sheetData>

</xml_diff>